<commit_message>
Atualiza sistema de declarações
</commit_message>
<xml_diff>
--- a/LISTA DE ALUNOS.xlsx
+++ b/LISTA DE ALUNOS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30317"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1893b7346536042/CESC/Dados alunos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="955" documentId="13_ncr:1_{4156C3C6-86C2-45D0-A343-A752AEC8871F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B2BF193-7C26-4B97-8F66-0479583D2910}"/>
+  <xr:revisionPtr revIDLastSave="957" documentId="13_ncr:1_{4156C3C6-86C2-45D0-A343-A752AEC8871F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D3ED554-F9C6-4BFE-BA6F-C61B97746F5F}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="3972" yWindow="3360" windowWidth="17280" windowHeight="8880" tabRatio="761" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4183" uniqueCount="1676">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4184" uniqueCount="1677">
   <si>
     <t>Unidade</t>
   </si>
@@ -4987,6 +4987,9 @@
   </si>
   <si>
     <t>Helena dos Santos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gerson </t>
   </si>
   <si>
     <t>Linha 3: exemplo de preenchimento</t>
@@ -5357,7 +5360,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="117">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -5653,56 +5656,38 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
-    <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
+    <cellStyle name="Hiperligação" xfId="2" builtinId="8"/>
     <cellStyle name="Hyperlink" xfId="3" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{3CB87C3B-3C31-4257-9DFA-F77E54F261B7}"/>
   </cellStyles>
   <dxfs count="54">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <sz val="9"/>
@@ -5838,6 +5823,18 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -6514,6 +6511,13 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <bottom style="thin">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
         <left style="thin">
           <color rgb="FFCCCCCC"/>
         </left>
@@ -6545,13 +6549,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color rgb="FFCCCCCC"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <font>
@@ -6586,6 +6583,36 @@
         <top/>
         <bottom/>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -6638,66 +6665,66 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{306DC3E5-E315-48F0-988E-C2B2CED54EF5}" name="Tabela35" displayName="Tabela35" ref="A1:AB254" totalsRowShown="0" headerRowDxfId="50" dataDxfId="48" headerRowBorderDxfId="49" tableBorderDxfId="47">
-  <autoFilter ref="A1:AB254" xr:uid="{E4A5C1DD-B238-4CCD-BCD0-1FE9F6D8442A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{306DC3E5-E315-48F0-988E-C2B2CED54EF5}" name="Tabela35" displayName="Tabela35" ref="A1:AB255" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46" headerRowBorderDxfId="44" tableBorderDxfId="45">
+  <autoFilter ref="A1:AB255" xr:uid="{E4A5C1DD-B238-4CCD-BCD0-1FE9F6D8442A}"/>
   <tableColumns count="28">
-    <tableColumn id="1" xr3:uid="{E42EC42B-46FD-4743-99E6-E9C6851F2FE6}" name="Aluno" dataDxfId="46"/>
-    <tableColumn id="29" xr3:uid="{6078CFA9-E6C9-4841-8147-AFEF7CF380C5}" name="Data de Nascimento" dataDxfId="45"/>
-    <tableColumn id="32" xr3:uid="{EFA272F8-3805-4A2D-8341-109210C81766}" name="Valor fixo" dataDxfId="44"/>
-    <tableColumn id="2" xr3:uid="{EE6B71EC-A5D4-4153-88B9-436B57EEB961}" name="Valor com desc" dataDxfId="43"/>
-    <tableColumn id="3" xr3:uid="{ADEC2FF3-1D7D-4817-A670-5826BC965C38}" name="Mês" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{20E5EDB3-7B52-4476-ABDE-1BE092EA23A7}" name="Renovação ou novo?" dataDxfId="41"/>
-    <tableColumn id="5" xr3:uid="{040624A1-5A2C-475F-9322-1E7EEA047982}" name="Unidade" dataDxfId="40"/>
-    <tableColumn id="6" xr3:uid="{49943602-11ED-4DAB-A2B9-8311BF8CE0DE}" name="Turma" dataDxfId="39"/>
-    <tableColumn id="7" xr3:uid="{9BF6A32E-FD32-4DEB-82E4-3B316BCA57E7}" name="Modalidade escolhida" dataDxfId="38"/>
-    <tableColumn id="8" xr3:uid="{511CADE1-AAB7-40A5-A7F7-D08BF05E216B}" name="E-mail" dataDxfId="37"/>
-    <tableColumn id="10" xr3:uid="{1470B8D6-17D9-4CB5-BA46-F7EBBC701BCC}" name="Nome responsável financeiro" dataDxfId="36"/>
-    <tableColumn id="28" xr3:uid="{5A37D809-53D3-4A30-BA12-FC65390A185E}" name="CPF" dataDxfId="35"/>
-    <tableColumn id="26" xr3:uid="{D5A43AE5-EC49-4897-BB16-C84DDAF8B41A}" name="Nome da Mãe" dataDxfId="34"/>
-    <tableColumn id="25" xr3:uid="{BD1532CD-F194-4C66-8B9E-3881C4D24F23}" name="Nome do Pai" dataDxfId="33"/>
-    <tableColumn id="12" xr3:uid="{CCECD66E-9216-4DB0-A606-F3B347A96AD4}" name="Telefone" dataDxfId="32"/>
-    <tableColumn id="27" xr3:uid="{27572104-3CD4-457E-BB09-17DB6C2D9700}" name="CEP" dataDxfId="31"/>
-    <tableColumn id="31" xr3:uid="{4D44B62C-0688-4EAA-9444-275FA0230736}" name="Endereço" dataDxfId="30"/>
-    <tableColumn id="30" xr3:uid="{4C268531-958C-489B-9DC2-B6A15C9A24F7}" name="numero" dataDxfId="29"/>
-    <tableColumn id="13" xr3:uid="{0B462660-AFBC-4E8C-B117-6C25785E80A0}" name="Contrato" dataDxfId="28"/>
-    <tableColumn id="14" xr3:uid="{B2903D32-D41B-4739-B52C-46A5672567F5}" name="Doc" dataDxfId="27"/>
-    <tableColumn id="15" xr3:uid="{17F7E6C9-D363-4797-BD37-3F0E03F9EBD0}" name="Asaas" dataDxfId="26"/>
-    <tableColumn id="16" xr3:uid="{06CE9C46-D781-48C6-93D6-92920BEEC34B}" name="Assinatura imagem" dataDxfId="25"/>
-    <tableColumn id="17" xr3:uid="{660597EB-81BA-4CFE-B067-A17BB8865800}" name="Data matricula" dataDxfId="24"/>
-    <tableColumn id="9" xr3:uid="{34C161C6-668B-4228-8DBD-000B67F9FB15}" name="Ficha Física" dataDxfId="23"/>
-    <tableColumn id="18" xr3:uid="{A58C020E-FEE4-4B20-89C1-844E859B7379}" name="Ativo?" dataDxfId="22"/>
-    <tableColumn id="19" xr3:uid="{A6ECECBB-C005-4FC4-923B-7F1E3845250A}" name="Link do doc" dataDxfId="21"/>
-    <tableColumn id="22" xr3:uid="{F61BBB7C-2966-4EA9-8D29-D0697BBE7C1F}" name="Observação" dataDxfId="20"/>
-    <tableColumn id="23" xr3:uid="{F8CDDB73-FF0B-4379-B236-AC526AF2C253}" name="CHECK MATRICULAS" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{E42EC42B-46FD-4743-99E6-E9C6851F2FE6}" name="Aluno" dataDxfId="43"/>
+    <tableColumn id="29" xr3:uid="{6078CFA9-E6C9-4841-8147-AFEF7CF380C5}" name="Data de Nascimento" dataDxfId="42"/>
+    <tableColumn id="32" xr3:uid="{EFA272F8-3805-4A2D-8341-109210C81766}" name="Valor fixo" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{EE6B71EC-A5D4-4153-88B9-436B57EEB961}" name="Valor com desc" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{ADEC2FF3-1D7D-4817-A670-5826BC965C38}" name="Mês" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{20E5EDB3-7B52-4476-ABDE-1BE092EA23A7}" name="Renovação ou novo?" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{040624A1-5A2C-475F-9322-1E7EEA047982}" name="Unidade" dataDxfId="37"/>
+    <tableColumn id="6" xr3:uid="{49943602-11ED-4DAB-A2B9-8311BF8CE0DE}" name="Turma" dataDxfId="36"/>
+    <tableColumn id="7" xr3:uid="{9BF6A32E-FD32-4DEB-82E4-3B316BCA57E7}" name="Modalidade escolhida" dataDxfId="35"/>
+    <tableColumn id="8" xr3:uid="{511CADE1-AAB7-40A5-A7F7-D08BF05E216B}" name="E-mail" dataDxfId="34"/>
+    <tableColumn id="10" xr3:uid="{1470B8D6-17D9-4CB5-BA46-F7EBBC701BCC}" name="Nome responsável financeiro" dataDxfId="33"/>
+    <tableColumn id="28" xr3:uid="{5A37D809-53D3-4A30-BA12-FC65390A185E}" name="CPF" dataDxfId="32"/>
+    <tableColumn id="26" xr3:uid="{D5A43AE5-EC49-4897-BB16-C84DDAF8B41A}" name="Nome da Mãe" dataDxfId="31"/>
+    <tableColumn id="25" xr3:uid="{BD1532CD-F194-4C66-8B9E-3881C4D24F23}" name="Nome do Pai" dataDxfId="30"/>
+    <tableColumn id="12" xr3:uid="{CCECD66E-9216-4DB0-A606-F3B347A96AD4}" name="Telefone" dataDxfId="29"/>
+    <tableColumn id="27" xr3:uid="{27572104-3CD4-457E-BB09-17DB6C2D9700}" name="CEP" dataDxfId="28"/>
+    <tableColumn id="31" xr3:uid="{4D44B62C-0688-4EAA-9444-275FA0230736}" name="Endereço" dataDxfId="27"/>
+    <tableColumn id="30" xr3:uid="{4C268531-958C-489B-9DC2-B6A15C9A24F7}" name="numero" dataDxfId="26"/>
+    <tableColumn id="13" xr3:uid="{0B462660-AFBC-4E8C-B117-6C25785E80A0}" name="Contrato" dataDxfId="25"/>
+    <tableColumn id="14" xr3:uid="{B2903D32-D41B-4739-B52C-46A5672567F5}" name="Doc" dataDxfId="24"/>
+    <tableColumn id="15" xr3:uid="{17F7E6C9-D363-4797-BD37-3F0E03F9EBD0}" name="Asaas" dataDxfId="23"/>
+    <tableColumn id="16" xr3:uid="{06CE9C46-D781-48C6-93D6-92920BEEC34B}" name="Assinatura imagem" dataDxfId="22"/>
+    <tableColumn id="17" xr3:uid="{660597EB-81BA-4CFE-B067-A17BB8865800}" name="Data matricula" dataDxfId="21"/>
+    <tableColumn id="9" xr3:uid="{34C161C6-668B-4228-8DBD-000B67F9FB15}" name="Ficha Física" dataDxfId="20"/>
+    <tableColumn id="18" xr3:uid="{A58C020E-FEE4-4B20-89C1-844E859B7379}" name="Ativo?" dataDxfId="19"/>
+    <tableColumn id="19" xr3:uid="{A6ECECBB-C005-4FC4-923B-7F1E3845250A}" name="Link do doc" dataDxfId="18"/>
+    <tableColumn id="22" xr3:uid="{F61BBB7C-2966-4EA9-8D29-D0697BBE7C1F}" name="Observação" dataDxfId="17"/>
+    <tableColumn id="23" xr3:uid="{F8CDDB73-FF0B-4379-B236-AC526AF2C253}" name="CHECK MATRICULAS" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA5002B6-9CF4-4812-BFF9-D24560D7988D}" name="Cancelamento" displayName="Cancelamento" ref="A2:F16" headerRowDxfId="18" headerRowBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA5002B6-9CF4-4812-BFF9-D24560D7988D}" name="Cancelamento" displayName="Cancelamento" ref="A2:F16" headerRowDxfId="13" headerRowBorderDxfId="12">
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{159DBC70-2DB3-4051-BEEE-0F283222906C}" name="Aluno"/>
     <tableColumn id="3" xr3:uid="{DD91A725-303E-4C2A-B780-2B3DB47EFE11}" name="Responsável"/>
     <tableColumn id="4" xr3:uid="{1EE1C561-D3FF-4AF1-94AB-949D5054E9B4}" name="Em dia"/>
-    <tableColumn id="5" xr3:uid="{B0131F87-3DEE-412B-8356-99068E45FA44}" name="Fase" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{B0131F87-3DEE-412B-8356-99068E45FA44}" name="Fase" dataDxfId="11"/>
     <tableColumn id="6" xr3:uid="{4B1C7395-48EA-4C90-AF38-2ECE85F81073}" name="Data de cancelamento"/>
-    <tableColumn id="7" xr3:uid="{D9B371B7-6695-4044-861F-921F9E507CA3}" name="Observações" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{D9B371B7-6695-4044-861F-921F9E507CA3}" name="Observações" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="Página1-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E3485996-CA2A-4BB0-AED0-8F37AA1E1E48}" name="Cancelamento3" displayName="Cancelamento3" ref="A2:G16" headerRowDxfId="14" dataDxfId="13" tableBorderDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E3485996-CA2A-4BB0-AED0-8F37AA1E1E48}" name="Cancelamento3" displayName="Cancelamento3" ref="A2:G16" headerRowDxfId="9" dataDxfId="8" tableBorderDxfId="7">
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{0907135F-365D-4466-9ECC-BC0BB331D168}" name="Aluno" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{EF8968E1-A123-4D64-B266-A15909BD7F0A}" name="Responsável" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{CE56CCDC-746C-46B5-A0F3-EE52CE258185}" name="Valor do acordo" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{56E430B1-1D41-4EEF-B8A6-776A77D16A09}" name="Parcelas" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{BE420054-ECBC-43A3-953D-EF77D43FCCF9}" name="data de vencimento" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{02B6F01C-82E7-41DD-A980-F0EC72C0BA79}" name="Foi feito novo contrato e assinado?" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{37C87BE4-1B71-4BE1-BABA-C3C3C2EB8D14}" name="Inicio da parcela" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{0907135F-365D-4466-9ECC-BC0BB331D168}" name="Aluno" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{EF8968E1-A123-4D64-B266-A15909BD7F0A}" name="Responsável" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{CE56CCDC-746C-46B5-A0F3-EE52CE258185}" name="Valor do acordo" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{56E430B1-1D41-4EEF-B8A6-776A77D16A09}" name="Parcelas" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{BE420054-ECBC-43A3-953D-EF77D43FCCF9}" name="data de vencimento" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{02B6F01C-82E7-41DD-A980-F0EC72C0BA79}" name="Foi feito novo contrato e assinado?" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{37C87BE4-1B71-4BE1-BABA-C3C3C2EB8D14}" name="Inicio da parcela" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="Página1-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6902,12 +6929,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F01DB8D-BC3C-4D77-BE59-D6F1AF6B0128}">
   <dimension ref="A1:I14"/>
-  <sheetFormatPr defaultRowHeight="13.2"/>
+  <sheetFormatPr defaultRowHeight="13.15"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.44140625" customWidth="1"/>
-    <col min="8" max="8" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.42578125" customWidth="1"/>
+    <col min="8" max="8" width="17.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -7078,35 +7105,35 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:AB401"/>
-  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="40.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.44140625" style="35" customWidth="1"/>
-    <col min="3" max="3" width="19.44140625" style="31" customWidth="1"/>
+    <col min="1" max="1" width="40.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" style="35" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" style="31" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="6.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.5546875" customWidth="1"/>
-    <col min="7" max="8" width="12.5546875" customWidth="1"/>
-    <col min="9" max="9" width="22.5546875" customWidth="1"/>
+    <col min="5" max="5" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" customWidth="1"/>
+    <col min="7" max="8" width="12.5703125" customWidth="1"/>
+    <col min="9" max="9" width="22.5703125" customWidth="1"/>
     <col min="10" max="10" width="35" style="36" customWidth="1"/>
-    <col min="11" max="11" width="43.44140625" style="30" customWidth="1"/>
-    <col min="12" max="12" width="19.44140625" customWidth="1"/>
-    <col min="13" max="14" width="43.44140625" customWidth="1"/>
-    <col min="15" max="15" width="15.44140625" customWidth="1"/>
-    <col min="16" max="16" width="15.44140625" style="29" customWidth="1"/>
-    <col min="17" max="17" width="15.44140625" style="30" customWidth="1"/>
-    <col min="18" max="19" width="15.44140625" customWidth="1"/>
-    <col min="20" max="20" width="12.5546875" customWidth="1"/>
-    <col min="21" max="21" width="14.44140625" customWidth="1"/>
-    <col min="22" max="22" width="20.5546875" customWidth="1"/>
-    <col min="23" max="24" width="16.5546875" customWidth="1"/>
+    <col min="11" max="11" width="43.42578125" style="30" customWidth="1"/>
+    <col min="12" max="12" width="19.42578125" customWidth="1"/>
+    <col min="13" max="14" width="43.42578125" customWidth="1"/>
+    <col min="15" max="15" width="15.42578125" customWidth="1"/>
+    <col min="16" max="16" width="15.42578125" style="29" customWidth="1"/>
+    <col min="17" max="17" width="15.42578125" style="30" customWidth="1"/>
+    <col min="18" max="19" width="15.42578125" customWidth="1"/>
+    <col min="20" max="20" width="12.5703125" customWidth="1"/>
+    <col min="21" max="21" width="14.42578125" customWidth="1"/>
+    <col min="22" max="22" width="20.5703125" customWidth="1"/>
+    <col min="23" max="24" width="16.5703125" customWidth="1"/>
     <col min="25" max="25" width="15" customWidth="1"/>
-    <col min="26" max="26" width="32.5546875" customWidth="1"/>
-    <col min="27" max="27" width="28.44140625" customWidth="1"/>
-    <col min="28" max="28" width="23.5546875" customWidth="1"/>
+    <col min="26" max="26" width="32.5703125" customWidth="1"/>
+    <col min="27" max="27" width="28.42578125" customWidth="1"/>
+    <col min="28" max="28" width="23.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="14.4">
+    <row r="1" spans="1:28" ht="14.45">
       <c r="A1" s="42" t="s">
         <v>39</v>
       </c>
@@ -25456,7 +25483,40 @@
       <c r="AA254" s="54"/>
       <c r="AB254" s="54"/>
     </row>
-    <row r="255" spans="1:28" ht="22.5" customHeight="1"/>
+    <row r="255" spans="1:28" ht="22.5" customHeight="1">
+      <c r="A255" s="109" t="s">
+        <v>1648</v>
+      </c>
+      <c r="B255" s="110">
+        <v>46231</v>
+      </c>
+      <c r="C255" s="111"/>
+      <c r="D255" s="112"/>
+      <c r="E255" s="109"/>
+      <c r="F255" s="109"/>
+      <c r="G255" s="109"/>
+      <c r="H255" s="109"/>
+      <c r="I255" s="109"/>
+      <c r="J255" s="113"/>
+      <c r="K255" s="114"/>
+      <c r="L255" s="109"/>
+      <c r="M255" s="109"/>
+      <c r="N255" s="109"/>
+      <c r="O255" s="109"/>
+      <c r="P255" s="115"/>
+      <c r="Q255" s="114"/>
+      <c r="R255" s="114"/>
+      <c r="S255" s="109"/>
+      <c r="T255" s="109"/>
+      <c r="U255" s="109"/>
+      <c r="V255" s="109"/>
+      <c r="W255" s="109"/>
+      <c r="X255" s="51"/>
+      <c r="Y255" s="109"/>
+      <c r="Z255" s="109"/>
+      <c r="AA255" s="109"/>
+      <c r="AB255" s="116"/>
+    </row>
     <row r="256" spans="1:28" ht="22.5" customHeight="1"/>
     <row r="257" ht="22.5" customHeight="1"/>
     <row r="258" ht="22.5" customHeight="1"/>
@@ -25615,15 +25675,15 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S2:U71 S72:T72 S73:U1048576">
-    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="50" priority="3" operator="equal">
       <formula>"Pendente"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V2:V1048576">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="49" priority="1" operator="equal">
       <formula>"Pendente"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="48" priority="2" operator="equal">
       <formula>"Não autorizado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -26061,19 +26121,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C57EAB1-5CCB-4D52-BFE8-5CC7FE7602FC}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultColWidth="15.5546875" defaultRowHeight="29.85" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="15.5703125" defaultRowHeight="29.85" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="34.5546875" customWidth="1"/>
-    <col min="2" max="2" width="22.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.5546875" customWidth="1"/>
-    <col min="4" max="4" width="18.44140625" style="30" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.44140625" customWidth="1"/>
-    <col min="6" max="6" width="19.44140625" customWidth="1"/>
+    <col min="1" max="1" width="34.5703125" customWidth="1"/>
+    <col min="2" max="2" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5703125" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" style="30" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.42578125" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="17.100000000000001" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="29.85" customHeight="1">
@@ -26081,34 +26141,34 @@
         <v>39</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>1650</v>
+        <v>1651</v>
       </c>
       <c r="D2" s="33" t="s">
-        <v>1651</v>
+        <v>1652</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1652</v>
+        <v>1653</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>1653</v>
+        <v>1654</v>
       </c>
       <c r="H2" s="8"/>
     </row>
     <row r="3" spans="1:8" ht="29.85" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="C3" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D3" s="32" t="s">
-        <v>1656</v>
+        <v>1657</v>
       </c>
       <c r="E3" s="10">
         <v>45729</v>
@@ -26118,7 +26178,7 @@
     </row>
     <row r="4" spans="1:8" ht="29.85" customHeight="1">
       <c r="A4" s="18" t="s">
-        <v>1657</v>
+        <v>1658</v>
       </c>
       <c r="B4" s="18" t="s">
         <v>1127</v>
@@ -26127,7 +26187,7 @@
         <v>77</v>
       </c>
       <c r="D4" s="34" t="s">
-        <v>1658</v>
+        <v>1659</v>
       </c>
       <c r="E4" s="21">
         <v>46097</v>
@@ -26184,7 +26244,7 @@
     </row>
     <row r="8" spans="1:8" ht="29.85" customHeight="1">
       <c r="A8" s="18" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>1413</v>
@@ -26209,7 +26269,7 @@
         <v>77</v>
       </c>
       <c r="D9" s="32" t="s">
-        <v>1656</v>
+        <v>1657</v>
       </c>
       <c r="E9" s="12">
         <v>46199</v>
@@ -26274,12 +26334,12 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D3:D5">
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Assinado">
+    <cfRule type="containsText" dxfId="15" priority="2" operator="containsText" text="Assinado">
       <formula>NOT(ISERROR(SEARCH("Assinado",D3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D9">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Assinado">
+    <cfRule type="containsText" dxfId="14" priority="1" operator="containsText" text="Assinado">
       <formula>NOT(ISERROR(SEARCH("Assinado",D9)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -26308,21 +26368,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F5626B0-8D8C-47DE-9EC8-B1C3DAE3BEDE}">
   <dimension ref="A1:I16"/>
-  <sheetFormatPr defaultColWidth="15.5546875" defaultRowHeight="29.85" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="15.5703125" defaultRowHeight="29.85" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="34.5546875" customWidth="1"/>
-    <col min="2" max="2" width="30.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.5703125" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.5546875" customWidth="1"/>
-    <col min="7" max="7" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.5703125" customWidth="1"/>
+    <col min="7" max="7" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="33.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="17.100000000000001" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="48" customHeight="1">
@@ -26330,22 +26390,22 @@
         <v>39</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="I2" t="s">
         <v>12</v>
@@ -26353,16 +26413,16 @@
     </row>
     <row r="3" spans="1:9" ht="29.85" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="C3" s="7">
         <v>3476</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>1665</v>
+        <v>1666</v>
       </c>
       <c r="E3" s="9">
         <v>20</v>
@@ -26372,12 +26432,12 @@
         <v>45748</v>
       </c>
       <c r="I3" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="29.85" customHeight="1">
       <c r="A4" s="18" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>1511</v>
@@ -26386,18 +26446,18 @@
         <v>1000</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>1668</v>
+        <v>1669</v>
       </c>
       <c r="E4" s="21"/>
       <c r="F4" s="22"/>
       <c r="G4" s="23"/>
       <c r="I4" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="29.85" customHeight="1">
       <c r="A5" s="6" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="7">
@@ -26408,30 +26468,30 @@
       <c r="F5" s="9"/>
       <c r="G5" s="13"/>
       <c r="I5" t="s">
-        <v>1671</v>
+        <v>1672</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="29.85" customHeight="1">
       <c r="A6" s="18" t="s">
-        <v>1672</v>
+        <v>1673</v>
       </c>
       <c r="B6" s="18"/>
       <c r="C6" s="19">
         <v>1800</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>1673</v>
+        <v>1674</v>
       </c>
       <c r="E6" s="21"/>
       <c r="F6" s="22"/>
       <c r="G6" s="23"/>
       <c r="I6" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="29.85" customHeight="1">
       <c r="A7" s="6" t="s">
-        <v>1675</v>
+        <v>1676</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>481</v>

</xml_diff>